<commit_message>
GUI fixes: data request text, classic export provider name, provider selector sync
- Remove '(typform data request)' text from download popup; link text now
  generic 'request your data' (valid for all providers, no 404)
- Fix classic export path log message: uses adapter display_name instead
  of hardcoded 'Perplexity' (was referring to Claude as Perplexity)
- Sync export-provider-select (page 2) with provider-select (page 1) on
  connect: getState() now returns provider; applyState() + connected
  handler sync both dropdowns + updateProviderUI()
- Fix 'Files are grouped like' -> 'Files are grouped the same way <provider>
  does for itself' (factually correct per-provider)
- Timer span uses white-space:nowrap to prevent seconds wrapping
- bridge.py: connected push payload includes provider field
- Rebuild dist/TotalRecalls.exe
</commit_message>
<xml_diff>
--- a/docs/AI Models Credentials.xlsx
+++ b/docs/AI Models Credentials.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\break\Projects\TotalRecalls\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3468BF4C-90B3-436E-8528-4DDD17D67615}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A860CA2A-11AE-42ED-8FD2-1F47A37D842D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="43395" yWindow="3495" windowWidth="9540" windowHeight="15555" xr2:uid="{7E254205-7D72-479A-B93B-5909398EDE61}"/>
   </bookViews>
@@ -83,7 +83,7 @@
     <t>breakwatercap.1@gmail.com</t>
   </si>
   <si>
-    <t>Bizard2024!!</t>
+    <t>Bizard2024!</t>
   </si>
 </sst>
 </file>

</xml_diff>